<commit_message>
feat: auth login + animated home + extractor v9 BILAN fix
</commit_message>
<xml_diff>
--- a/data/processed/data_bancaire_senegal_2015_2022.xlsx
+++ b/data/processed/data_bancaire_senegal_2015_2022.xlsx
@@ -2669,8 +2669,12 @@
       <c r="D20" t="n">
         <v>171288</v>
       </c>
-      <c r="E20" t="inlineStr"/>
-      <c r="F20" t="inlineStr"/>
+      <c r="E20" t="n">
+        <v>302954</v>
+      </c>
+      <c r="F20" t="n">
+        <v>174606</v>
+      </c>
       <c r="G20" t="n">
         <v>27531</v>
       </c>
@@ -2845,8 +2849,12 @@
       <c r="D21" t="n">
         <v>209097</v>
       </c>
-      <c r="E21" t="inlineStr"/>
-      <c r="F21" t="inlineStr"/>
+      <c r="E21" t="n">
+        <v>357558</v>
+      </c>
+      <c r="F21" t="n">
+        <v>232315</v>
+      </c>
       <c r="G21" t="n">
         <v>32601</v>
       </c>
@@ -4099,8 +4107,12 @@
       <c r="D33" t="n">
         <v>376905</v>
       </c>
-      <c r="E33" t="inlineStr"/>
-      <c r="F33" t="inlineStr"/>
+      <c r="E33" t="n">
+        <v>532817</v>
+      </c>
+      <c r="F33" t="n">
+        <v>352184</v>
+      </c>
       <c r="G33" t="n">
         <v>50088</v>
       </c>
@@ -4277,8 +4289,12 @@
       <c r="D34" t="n">
         <v>419539</v>
       </c>
-      <c r="E34" t="inlineStr"/>
-      <c r="F34" t="inlineStr"/>
+      <c r="E34" t="n">
+        <v>564277</v>
+      </c>
+      <c r="F34" t="n">
+        <v>404621</v>
+      </c>
       <c r="G34" t="n">
         <v>52686</v>
       </c>
@@ -5109,8 +5125,12 @@
       <c r="D41" t="n">
         <v>301622</v>
       </c>
-      <c r="E41" t="inlineStr"/>
-      <c r="F41" t="inlineStr"/>
+      <c r="E41" t="n">
+        <v>557927</v>
+      </c>
+      <c r="F41" t="n">
+        <v>430973</v>
+      </c>
       <c r="G41" t="n">
         <v>67569</v>
       </c>
@@ -5287,8 +5307,12 @@
       <c r="D42" t="n">
         <v>324279</v>
       </c>
-      <c r="E42" t="inlineStr"/>
-      <c r="F42" t="inlineStr"/>
+      <c r="E42" t="n">
+        <v>668837</v>
+      </c>
+      <c r="F42" t="n">
+        <v>563492</v>
+      </c>
       <c r="G42" t="n">
         <v>64191</v>
       </c>
@@ -6109,8 +6133,12 @@
       <c r="D49" t="n">
         <v>458187</v>
       </c>
-      <c r="E49" t="inlineStr"/>
-      <c r="F49" t="inlineStr"/>
+      <c r="E49" t="n">
+        <v>580532</v>
+      </c>
+      <c r="F49" t="n">
+        <v>388378</v>
+      </c>
       <c r="G49" t="n">
         <v>63512</v>
       </c>
@@ -6279,8 +6307,12 @@
       <c r="D50" t="n">
         <v>563859</v>
       </c>
-      <c r="E50" t="inlineStr"/>
-      <c r="F50" t="inlineStr"/>
+      <c r="E50" t="n">
+        <v>735887</v>
+      </c>
+      <c r="F50" t="n">
+        <v>504514</v>
+      </c>
       <c r="G50" t="n">
         <v>68034</v>
       </c>
@@ -7093,8 +7125,12 @@
       <c r="D57" t="n">
         <v>147251</v>
       </c>
-      <c r="E57" t="inlineStr"/>
-      <c r="F57" t="inlineStr"/>
+      <c r="E57" t="n">
+        <v>332836</v>
+      </c>
+      <c r="F57" t="n">
+        <v>170102</v>
+      </c>
       <c r="G57" t="n">
         <v>36763</v>
       </c>
@@ -7271,8 +7307,12 @@
       <c r="D58" t="n">
         <v>163570</v>
       </c>
-      <c r="E58" t="inlineStr"/>
-      <c r="F58" t="inlineStr"/>
+      <c r="E58" t="n">
+        <v>400545</v>
+      </c>
+      <c r="F58" t="n">
+        <v>181334</v>
+      </c>
       <c r="G58" t="n">
         <v>37216</v>
       </c>
@@ -8543,8 +8583,12 @@
       <c r="D70" t="n">
         <v>97783</v>
       </c>
-      <c r="E70" t="inlineStr"/>
-      <c r="F70" t="inlineStr"/>
+      <c r="E70" t="n">
+        <v>195994</v>
+      </c>
+      <c r="F70" t="n">
+        <v>134082</v>
+      </c>
       <c r="G70" t="n">
         <v>-80102</v>
       </c>
@@ -8717,8 +8761,12 @@
       <c r="D71" t="n">
         <v>84661</v>
       </c>
-      <c r="E71" t="inlineStr"/>
-      <c r="F71" t="inlineStr"/>
+      <c r="E71" t="n">
+        <v>160540</v>
+      </c>
+      <c r="F71" t="n">
+        <v>138439</v>
+      </c>
       <c r="G71" t="n">
         <v>-86821</v>
       </c>
@@ -9355,8 +9403,12 @@
       <c r="D76" t="n">
         <v>72020</v>
       </c>
-      <c r="E76" t="inlineStr"/>
-      <c r="F76" t="inlineStr"/>
+      <c r="E76" t="n">
+        <v>149665</v>
+      </c>
+      <c r="F76" t="n">
+        <v>81891</v>
+      </c>
       <c r="G76" t="n">
         <v>5994</v>
       </c>
@@ -9531,8 +9583,12 @@
       <c r="D77" t="n">
         <v>118893</v>
       </c>
-      <c r="E77" t="inlineStr"/>
-      <c r="F77" t="inlineStr"/>
+      <c r="E77" t="n">
+        <v>208152</v>
+      </c>
+      <c r="F77" t="n">
+        <v>137657</v>
+      </c>
       <c r="G77" t="n">
         <v>30500</v>
       </c>
@@ -10359,8 +10415,12 @@
       <c r="D84" t="n">
         <v>754858</v>
       </c>
-      <c r="E84" t="inlineStr"/>
-      <c r="F84" t="inlineStr"/>
+      <c r="E84" t="n">
+        <v>1183343</v>
+      </c>
+      <c r="F84" t="n">
+        <v>969295</v>
+      </c>
       <c r="G84" t="n">
         <v>124305</v>
       </c>
@@ -10537,8 +10597,12 @@
       <c r="D85" t="n">
         <v>871980</v>
       </c>
-      <c r="E85" t="inlineStr"/>
-      <c r="F85" t="inlineStr"/>
+      <c r="E85" t="n">
+        <v>1350783</v>
+      </c>
+      <c r="F85" t="n">
+        <v>1102891</v>
+      </c>
       <c r="G85" t="n">
         <v>138544</v>
       </c>
@@ -11809,8 +11873,12 @@
       <c r="D96" t="n">
         <v>155004</v>
       </c>
-      <c r="E96" t="inlineStr"/>
-      <c r="F96" t="inlineStr"/>
+      <c r="E96" t="n">
+        <v>244137</v>
+      </c>
+      <c r="F96" t="n">
+        <v>146641</v>
+      </c>
       <c r="G96" t="n">
         <v>32347</v>
       </c>
@@ -11987,8 +12055,12 @@
       <c r="D97" t="n">
         <v>178816</v>
       </c>
-      <c r="E97" t="inlineStr"/>
-      <c r="F97" t="inlineStr"/>
+      <c r="E97" t="n">
+        <v>286564</v>
+      </c>
+      <c r="F97" t="n">
+        <v>182680</v>
+      </c>
       <c r="G97" t="n">
         <v>35039</v>
       </c>
@@ -13451,8 +13523,12 @@
       <c r="D110" t="n">
         <v>46613</v>
       </c>
-      <c r="E110" t="inlineStr"/>
-      <c r="F110" t="inlineStr"/>
+      <c r="E110" t="n">
+        <v>227393</v>
+      </c>
+      <c r="F110" t="n">
+        <v>187753</v>
+      </c>
       <c r="G110" t="n">
         <v>28466</v>
       </c>
@@ -13627,8 +13703,12 @@
       <c r="D111" t="n">
         <v>106858</v>
       </c>
-      <c r="E111" t="inlineStr"/>
-      <c r="F111" t="inlineStr"/>
+      <c r="E111" t="n">
+        <v>278271</v>
+      </c>
+      <c r="F111" t="n">
+        <v>237285</v>
+      </c>
       <c r="G111" t="n">
         <v>31126</v>
       </c>
@@ -14449,8 +14529,12 @@
       <c r="D118" t="n">
         <v>352174</v>
       </c>
-      <c r="E118" t="inlineStr"/>
-      <c r="F118" t="inlineStr"/>
+      <c r="E118" t="n">
+        <v>832177</v>
+      </c>
+      <c r="F118" t="n">
+        <v>543241</v>
+      </c>
       <c r="G118" t="n">
         <v>52922</v>
       </c>
@@ -14623,8 +14707,12 @@
       <c r="D119" t="n">
         <v>387406</v>
       </c>
-      <c r="E119" t="inlineStr"/>
-      <c r="F119" t="inlineStr"/>
+      <c r="E119" t="n">
+        <v>965987</v>
+      </c>
+      <c r="F119" t="n">
+        <v>617763</v>
+      </c>
       <c r="G119" t="n">
         <v>2930</v>
       </c>
@@ -15433,8 +15521,12 @@
       <c r="D126" t="n">
         <v>75504</v>
       </c>
-      <c r="E126" t="inlineStr"/>
-      <c r="F126" t="inlineStr"/>
+      <c r="E126" t="n">
+        <v>121857</v>
+      </c>
+      <c r="F126" t="n">
+        <v>106562</v>
+      </c>
       <c r="G126" t="n">
         <v>12064</v>
       </c>
@@ -15609,8 +15701,12 @@
       <c r="D127" t="n">
         <v>116355</v>
       </c>
-      <c r="E127" t="inlineStr"/>
-      <c r="F127" t="inlineStr"/>
+      <c r="E127" t="n">
+        <v>309181</v>
+      </c>
+      <c r="F127" t="n">
+        <v>251111</v>
+      </c>
       <c r="G127" t="n">
         <v>14193</v>
       </c>
@@ -16413,8 +16509,12 @@
       <c r="D134" t="n">
         <v>276424</v>
       </c>
-      <c r="E134" t="inlineStr"/>
-      <c r="F134" t="inlineStr"/>
+      <c r="E134" t="n">
+        <v>368520</v>
+      </c>
+      <c r="F134" t="n">
+        <v>266113</v>
+      </c>
       <c r="G134" t="n">
         <v>23799</v>
       </c>
@@ -16591,8 +16691,12 @@
       <c r="D135" t="n">
         <v>288146</v>
       </c>
-      <c r="E135" t="inlineStr"/>
-      <c r="F135" t="inlineStr"/>
+      <c r="E135" t="n">
+        <v>405932</v>
+      </c>
+      <c r="F135" t="n">
+        <v>296149</v>
+      </c>
       <c r="G135" t="n">
         <v>23355</v>
       </c>
@@ -17201,8 +17305,12 @@
       <c r="D140" t="n">
         <v>26423</v>
       </c>
-      <c r="E140" t="inlineStr"/>
-      <c r="F140" t="inlineStr"/>
+      <c r="E140" t="n">
+        <v>40730</v>
+      </c>
+      <c r="F140" t="n">
+        <v>18781</v>
+      </c>
       <c r="G140" t="n">
         <v>9887</v>
       </c>
@@ -17379,8 +17487,12 @@
       <c r="D141" t="n">
         <v>36794</v>
       </c>
-      <c r="E141" t="inlineStr"/>
-      <c r="F141" t="inlineStr"/>
+      <c r="E141" t="n">
+        <v>57945</v>
+      </c>
+      <c r="F141" t="n">
+        <v>37046</v>
+      </c>
       <c r="G141" t="n">
         <v>10912</v>
       </c>
@@ -18685,8 +18797,12 @@
       <c r="D152" t="n">
         <v>367558</v>
       </c>
-      <c r="E152" t="inlineStr"/>
-      <c r="F152" t="inlineStr"/>
+      <c r="E152" t="n">
+        <v>643814</v>
+      </c>
+      <c r="F152" t="n">
+        <v>458251</v>
+      </c>
       <c r="G152" t="n">
         <v>37030</v>
       </c>
@@ -18857,8 +18973,12 @@
       <c r="D153" t="n">
         <v>464870</v>
       </c>
-      <c r="E153" t="inlineStr"/>
-      <c r="F153" t="inlineStr"/>
+      <c r="E153" t="n">
+        <v>838601</v>
+      </c>
+      <c r="F153" t="n">
+        <v>626552</v>
+      </c>
       <c r="G153" t="n">
         <v>50247</v>
       </c>
@@ -19679,8 +19799,12 @@
       <c r="D160" t="n">
         <v>664236</v>
       </c>
-      <c r="E160" t="inlineStr"/>
-      <c r="F160" t="inlineStr"/>
+      <c r="E160" t="n">
+        <v>1103875</v>
+      </c>
+      <c r="F160" t="n">
+        <v>914208</v>
+      </c>
       <c r="G160" t="n">
         <v>118677</v>
       </c>
@@ -19857,8 +19981,12 @@
       <c r="D161" t="n">
         <v>814220</v>
       </c>
-      <c r="E161" t="inlineStr"/>
-      <c r="F161" t="inlineStr"/>
+      <c r="E161" t="n">
+        <v>1337613</v>
+      </c>
+      <c r="F161" t="n">
+        <v>1057130</v>
+      </c>
       <c r="G161" t="n">
         <v>104951</v>
       </c>
@@ -20659,8 +20787,12 @@
       <c r="D168" t="n">
         <v>119030</v>
       </c>
-      <c r="E168" t="inlineStr"/>
-      <c r="F168" t="inlineStr"/>
+      <c r="E168" t="n">
+        <v>365046</v>
+      </c>
+      <c r="F168" t="n">
+        <v>252497</v>
+      </c>
       <c r="G168" t="n">
         <v>42109</v>
       </c>
@@ -20835,8 +20967,12 @@
       <c r="D169" t="n">
         <v>115693</v>
       </c>
-      <c r="E169" t="inlineStr"/>
-      <c r="F169" t="inlineStr"/>
+      <c r="E169" t="n">
+        <v>454020</v>
+      </c>
+      <c r="F169" t="n">
+        <v>256812</v>
+      </c>
       <c r="G169" t="n">
         <v>41917</v>
       </c>

</xml_diff>